<commit_message>
fix(excel): clarify live today inquiries vs cartable status and include bank trace IDs
</commit_message>
<xml_diff>
--- a/گزارش_جامع_استعلام_چک_ها_۱۴۰۵۰۶۱۵.xlsx
+++ b/گزارش_جامع_استعلام_چک_ها_۱۴۰۵۰۶۱۵.xlsx
@@ -219,10 +219,10 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -613,13 +613,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="119" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="29" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="82" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -635,7 +635,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>سامانه صیاد پرو ۳.۱ | تاریخ تهیه گزارش: 1405/06/15 ساعت 09:33:37 | منبع داده: درگاه رسمی بانک مرکزی و بانک پاسارگاد</t>
+          <t>سامانه صیاد پرو ۳.۱ | تاریخ تهیه گزارش: 1405/06/15 ساعت 16:05:36 | منبع داده: درگاه رسمی بانک مرکزی و بانک پاسارگاد</t>
         </is>
       </c>
     </row>
@@ -785,11 +785,11 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>استعلام‌های موفق لحظه‌ای درگاه</t>
+          <t>استعلام‌های زنده و بروز امروز درگاه</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
@@ -798,18 +798,18 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>استعلام مستقیم موفق از وب‌سرویس پاسارگاد امروز</t>
+          <t>استعلام مستقیم موفق از وب‌سرویس بانک پاسارگاد در تاریخ امروز با کد رهگیری زنده</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>چک‌های با حفظ سابقه معتبر</t>
+          <t>چک‌های با حفظ تاریخچه معتبر قبلی</t>
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
@@ -818,18 +818,18 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>حفظ ارقام معتبر پیشین بر اساس پایگاه داده</t>
+          <t>حفظ ارقام معتبر آخرین استعلام موفق (برای جلوگیری از صفر شدن داده‌ها)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>چک‌های تسویه یا سررسید گذشته</t>
+          <t>چک‌های خارج از کارتابل / عدم دسترسی</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
@@ -838,211 +838,231 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>سررسید گذشته و تسویه‌شده خارج از کارتابل</t>
+          <t>عدم حضور چک در کارتابل ۹ دارنده در استعلام گروهی امروز</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
+          <t>چک‌های سررسید گذشته و منقضی</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>فقره</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>سررسید گذشته و تسویه‌شده خارج از چرخه بانکی جاری</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
           <t>اسناد معاف از استعلام صیادی</t>
         </is>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B15" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>فقره</t>
         </is>
       </c>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>سفته‌ها و اسناد ضمانتی فاقد شناسه ۱۶ رقمی صیاد</t>
         </is>
       </c>
     </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>توزیع وضعیت رنگ اعتباری بانک مرکزی (CBI)</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>رنگ اعتباری</t>
         </is>
       </c>
-      <c r="B17" s="15" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>تعداد مشتریان</t>
         </is>
       </c>
-      <c r="C17" s="15" t="inlineStr">
+      <c r="C18" s="15" t="inlineStr">
         <is>
           <t>درصد از کل</t>
         </is>
       </c>
-      <c r="D17" s="15" t="inlineStr">
+      <c r="D18" s="15" t="inlineStr">
         <is>
           <t>ارزیابی ریسک</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>سفید (خوش‌حساب بدون برگشتی)</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="n">
-        <v>36</v>
-      </c>
-      <c r="C18" s="16" t="n">
-        <v>0.6923076923076923</v>
-      </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>کمترین ریسک اعتباری، فاقد هرگونه سوءاثر در سیستم بانکی</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>قرمز (دارای چک برگشتی فعال)</t>
+          <t>سفید (خوش‌حساب بدون برگشتی)</t>
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="C19" s="17" t="n">
-        <v>0.2692307692307692</v>
+        <v>36</v>
+      </c>
+      <c r="C19" s="16" t="n">
+        <v>0.6923076923076923</v>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>ریسک بالا؛ دارای چک برگشتی رفع سوءاثر نشده در شبکه بانکی</t>
+          <t>کمترین ریسک اعتباری، فاقد هرگونه سوءاثر در سیستم بانکی</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
+          <t>قرمز (دارای چک برگشتی فعال)</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="C20" s="17" t="n">
+        <v>0.2692307692307692</v>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>ریسک بالا؛ دارای چک برگشتی رفع سوءاثر نشده در شبکه بانکی</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
           <t>قهوه‌ای (سابقه چک‌های متعدد)</t>
         </is>
       </c>
-      <c r="B20" s="9" t="n">
+      <c r="B21" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="C20" s="16" t="n">
+      <c r="C21" s="16" t="n">
         <v>0.03846153846153846</v>
       </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>هشدار؛ سابقه چک‌های برگشتی مکرر یا حجم بالای نکول</t>
         </is>
       </c>
     </row>
-    <row r="21"/>
-    <row r="22">
-      <c r="A22" s="14" t="inlineStr">
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>ماتریس دوبعدی تحلیل ریسک اعتباری (Fintech Risk Matrix)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="15" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>رده ریسک مشتریان</t>
         </is>
       </c>
-      <c r="B23" s="15" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>تعداد مشتری</t>
         </is>
       </c>
-      <c r="C23" s="15" t="inlineStr">
+      <c r="C24" s="15" t="inlineStr">
         <is>
           <t>مجموع مبالغ تعهدات (ریال)</t>
         </is>
       </c>
-      <c r="D23" s="15" t="inlineStr">
+      <c r="D24" s="15" t="inlineStr">
         <is>
           <t>راهبرد پیشنهادی وصول و تعامل</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>ستاره‌ها (پرتراکنش و کم‌ریسک)</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="n">
-        <v>17</v>
-      </c>
-      <c r="C24" s="13" t="n">
-        <v>305440000000</v>
-      </c>
-      <c r="D24" s="11" t="inlineStr">
-        <is>
-          <t>توسعه همکاری و اعطای حداکثر تسهیلات و اعتبار تجاری</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>فرصت‌ها (کم‌تراکنش و کم‌ریسک)</t>
+          <t>ستاره‌ها (پرتراکنش و کم‌ریسک)</t>
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C25" s="12" t="n">
-        <v>29920000000</v>
+        <v>305440000000</v>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>افزایش حجم تراکنش و تشویق به همکاری بیشتر</t>
+          <t>توسعه همکاری و اعطای حداکثر تسهیلات و اعتبار تجاری</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>تحت نظر (پرریسک با مبالغ خرد)</t>
+          <t>فرصت‌ها (کم‌تراکنش و کم‌ریسک)</t>
         </is>
       </c>
       <c r="B26" s="9" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="C26" s="13" t="n">
-        <v>13265000000</v>
+        <v>29920000000</v>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>کنترل مستمر و پایش وصولی‌ها قبل از سررسید</t>
+          <t>افزایش حجم تراکنش و تشویق به همکاری بیشتر</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
+          <t>تحت نظر (پرریسک با مبالغ خرد)</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C27" s="12" t="n">
+        <v>13265000000</v>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>کنترل مستمر و پایش وصولی‌ها قبل از سررسید</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
           <t>بحرانی (پرریسک با تعهدات سنگین)</t>
         </is>
       </c>
-      <c r="B27" s="5" t="n">
+      <c r="B28" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="C27" s="12" t="n">
+      <c r="C28" s="13" t="n">
         <v>134700000000</v>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D28" s="11" t="inlineStr">
         <is>
           <t>اولویت فوری وصول؛ توقف پذیرش چک جدید و پیگیری حقوقی</t>
         </is>
@@ -1050,10 +1070,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A17:D17"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A23:D23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1080,12 +1100,12 @@
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="40" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="31" customWidth="1" min="12" max="12"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
     <col width="25" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
     <col width="23" customWidth="1" min="16" max="16"/>
-    <col width="65" customWidth="1" min="17" max="17"/>
+    <col width="109" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1298,7 +1318,7 @@
       </c>
       <c r="L3" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M3" s="12" t="n">
@@ -1317,7 +1337,7 @@
       </c>
       <c r="Q3" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:48 (کد پیگیری: 49685355323952)</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1395,7 @@
       </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M4" s="13" t="n">
@@ -1394,7 +1414,7 @@
       </c>
       <c r="Q4" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:48 (کد پیگیری: 49685355351830)</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1472,7 @@
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M5" s="12" t="n">
@@ -1471,7 +1491,7 @@
       </c>
       <c r="Q5" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:23 (کد پیگیری: 49685355298096)</t>
         </is>
       </c>
     </row>
@@ -1529,7 +1549,7 @@
       </c>
       <c r="L6" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M6" s="13" t="n">
@@ -1548,7 +1568,7 @@
       </c>
       <c r="Q6" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:52 (کد پیگیری: 49685355310602)</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1626,7 @@
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M7" s="12" t="n">
@@ -1625,7 +1645,7 @@
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:32 (کد پیگیری: 49685355323278)</t>
         </is>
       </c>
     </row>
@@ -1683,7 +1703,7 @@
       </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M8" s="13" t="n">
@@ -1702,7 +1722,7 @@
       </c>
       <c r="Q8" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:42 (کد پیگیری: 49685355308538)</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1776,7 @@
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M9" s="12" t="n">
@@ -1771,7 +1791,7 @@
       <c r="P9" s="6" t="inlineStr"/>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1849,7 @@
       </c>
       <c r="L10" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M10" s="13" t="n">
@@ -1848,7 +1868,7 @@
       </c>
       <c r="Q10" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:33 (کد پیگیری: 49685355296282)</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1991,7 @@
       </c>
       <c r="L12" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M12" s="13" t="n">
@@ -1990,7 +2010,7 @@
       </c>
       <c r="Q12" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:44 (کد پیگیری: 49685355304697)</t>
         </is>
       </c>
     </row>
@@ -2048,7 +2068,7 @@
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M13" s="12" t="n">
@@ -2067,7 +2087,7 @@
       </c>
       <c r="Q13" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:18 (کد پیگیری: 49685355310930)</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2145,7 @@
       </c>
       <c r="L14" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M14" s="13" t="n">
@@ -2144,7 +2164,7 @@
       </c>
       <c r="Q14" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:46 (کد پیگیری: 49685355335081)</t>
         </is>
       </c>
     </row>
@@ -2202,7 +2222,7 @@
       </c>
       <c r="L15" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M15" s="12" t="n">
@@ -2221,7 +2241,7 @@
       </c>
       <c r="Q15" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:22 (کد پیگیری: 49685355346621)</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2299,7 @@
       </c>
       <c r="L16" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M16" s="13" t="n">
@@ -2298,7 +2318,7 @@
       </c>
       <c r="Q16" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:22 (کد پیگیری: 49685355318256)</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2376,7 @@
       </c>
       <c r="L17" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M17" s="12" t="n">
@@ -2375,7 +2395,7 @@
       </c>
       <c r="Q17" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:03 (کد پیگیری: 49685355280874)</t>
         </is>
       </c>
     </row>
@@ -2433,7 +2453,7 @@
       </c>
       <c r="L18" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M18" s="13" t="n">
@@ -2452,7 +2472,7 @@
       </c>
       <c r="Q18" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:40 (کد پیگیری: 49685355308517)</t>
         </is>
       </c>
     </row>
@@ -2510,7 +2530,7 @@
       </c>
       <c r="L19" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M19" s="12" t="n">
@@ -2529,7 +2549,7 @@
       </c>
       <c r="Q19" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:14 (کد پیگیری: 49685355312796)</t>
         </is>
       </c>
     </row>
@@ -2587,7 +2607,7 @@
       </c>
       <c r="L20" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M20" s="13" t="n">
@@ -2606,7 +2626,7 @@
       </c>
       <c r="Q20" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:19 (کد پیگیری: 49685355346604)</t>
         </is>
       </c>
     </row>
@@ -2664,7 +2684,7 @@
       </c>
       <c r="L21" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M21" s="12" t="n">
@@ -2683,7 +2703,7 @@
       </c>
       <c r="Q21" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:37 (کد پیگیری: 49685355357612)</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2761,7 @@
       </c>
       <c r="L22" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M22" s="13" t="n">
@@ -2760,7 +2780,7 @@
       </c>
       <c r="Q22" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:43 (کد پیگیری: 49685355342484)</t>
         </is>
       </c>
     </row>
@@ -2818,7 +2838,7 @@
       </c>
       <c r="L23" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M23" s="12" t="n">
@@ -2837,7 +2857,7 @@
       </c>
       <c r="Q23" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:47 (کد پیگیری: 49685355345990)</t>
         </is>
       </c>
     </row>
@@ -2895,7 +2915,7 @@
       </c>
       <c r="L24" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M24" s="13" t="n">
@@ -2914,7 +2934,7 @@
       </c>
       <c r="Q24" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:20:59 (کد پیگیری: 49685355276391)</t>
         </is>
       </c>
     </row>
@@ -2972,7 +2992,7 @@
       </c>
       <c r="L25" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M25" s="12" t="n">
@@ -2991,7 +3011,7 @@
       </c>
       <c r="Q25" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:47 (کد پیگیری: 49685355304731)</t>
         </is>
       </c>
     </row>
@@ -3049,7 +3069,7 @@
       </c>
       <c r="L26" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M26" s="13" t="n">
@@ -3068,7 +3088,7 @@
       </c>
       <c r="Q26" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:21 (کد پیگیری: 49685355324524)</t>
         </is>
       </c>
     </row>
@@ -3126,7 +3146,7 @@
       </c>
       <c r="L27" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M27" s="12" t="n">
@@ -3145,7 +3165,7 @@
       </c>
       <c r="Q27" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:20:50 (کد پیگیری: 49685355280295)</t>
         </is>
       </c>
     </row>
@@ -3203,7 +3223,7 @@
       </c>
       <c r="L28" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M28" s="13" t="n">
@@ -3222,7 +3242,7 @@
       </c>
       <c r="Q28" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:17 (کد پیگیری: 49685355297086)</t>
         </is>
       </c>
     </row>
@@ -3280,7 +3300,7 @@
       </c>
       <c r="L29" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M29" s="12" t="n">
@@ -3299,7 +3319,7 @@
       </c>
       <c r="Q29" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:59 (کد پیگیری: 49685355335727)</t>
         </is>
       </c>
     </row>
@@ -3353,7 +3373,7 @@
       </c>
       <c r="L30" s="11" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M30" s="13" t="n">
@@ -3368,7 +3388,7 @@
       <c r="P30" s="10" t="inlineStr"/>
       <c r="Q30" s="11" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -3426,7 +3446,7 @@
       </c>
       <c r="L31" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M31" s="12" t="n">
@@ -3445,7 +3465,7 @@
       </c>
       <c r="Q31" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:02 (کد پیگیری: 49685355310724)</t>
         </is>
       </c>
     </row>
@@ -3503,7 +3523,7 @@
       </c>
       <c r="L32" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M32" s="13" t="n">
@@ -3522,7 +3542,7 @@
       </c>
       <c r="Q32" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:04 (کد پیگیری: 49685355336236)</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3600,7 @@
       </c>
       <c r="L33" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M33" s="12" t="n">
@@ -3599,7 +3619,7 @@
       </c>
       <c r="Q33" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:29 (کد پیگیری: 49685355348704)</t>
         </is>
       </c>
     </row>
@@ -3653,7 +3673,7 @@
       </c>
       <c r="L34" s="11" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M34" s="13" t="n">
@@ -3668,7 +3688,7 @@
       <c r="P34" s="10" t="inlineStr"/>
       <c r="Q34" s="11" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -3726,7 +3746,7 @@
       </c>
       <c r="L35" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M35" s="12" t="n">
@@ -3745,7 +3765,7 @@
       </c>
       <c r="Q35" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:16 (کد پیگیری: 49685355280999)</t>
         </is>
       </c>
     </row>
@@ -3803,7 +3823,7 @@
       </c>
       <c r="L36" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M36" s="13" t="n">
@@ -3822,7 +3842,7 @@
       </c>
       <c r="Q36" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:54 (کد پیگیری: 49685355305264)</t>
         </is>
       </c>
     </row>
@@ -3880,7 +3900,7 @@
       </c>
       <c r="L37" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M37" s="12" t="n">
@@ -3899,7 +3919,7 @@
       </c>
       <c r="Q37" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:25 (کد پیگیری: 49685355351542)</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3977,7 @@
       </c>
       <c r="L38" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M38" s="13" t="n">
@@ -3976,7 +3996,7 @@
       </c>
       <c r="Q38" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:40 (کد پیگیری: 49685355351224)</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4050,7 @@
       </c>
       <c r="L39" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M39" s="12" t="n">
@@ -4049,7 +4069,7 @@
       </c>
       <c r="Q39" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:36 (کد پیگیری: 49685355318403)</t>
         </is>
       </c>
     </row>
@@ -4107,7 +4127,7 @@
       </c>
       <c r="L40" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M40" s="13" t="n">
@@ -4126,7 +4146,7 @@
       </c>
       <c r="Q40" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:25 (کد پیگیری: 49685355320730)</t>
         </is>
       </c>
     </row>
@@ -4184,7 +4204,7 @@
       </c>
       <c r="L41" s="7" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M41" s="12" t="n">
@@ -4199,7 +4219,7 @@
       <c r="P41" s="6" t="inlineStr"/>
       <c r="Q41" s="7" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4292,7 @@
       <c r="P42" s="10" t="inlineStr"/>
       <c r="Q42" s="11" t="inlineStr">
         <is>
-          <t>سررسید چک در تاریخ 1405/05/28 منقضی شده و از کارتابل خارج است</t>
+          <t>سررسید چک در تاریخ 1405/05/28 منقضی شده و از کارتابل جاری خارج است</t>
         </is>
       </c>
     </row>
@@ -4330,7 +4350,7 @@
       </c>
       <c r="L43" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>حفظ تاریخچه معتبر قبلی</t>
         </is>
       </c>
       <c r="M43" s="12" t="n">
@@ -4349,7 +4369,7 @@
       </c>
       <c r="Q43" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>عدم حضور در کارتابل امروز؛ حفظ آخرین استعلام معتبر (2026-09-05 08:43:51) (کد پیگیری قبلی: 49682942030012)</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4427,7 @@
       </c>
       <c r="L44" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M44" s="13" t="n">
@@ -4426,7 +4446,7 @@
       </c>
       <c r="Q44" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:32 (کد پیگیری: 49685355303590)</t>
         </is>
       </c>
     </row>
@@ -4484,7 +4504,7 @@
       </c>
       <c r="L45" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M45" s="12" t="n">
@@ -4503,7 +4523,7 @@
       </c>
       <c r="Q45" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:11 (کد پیگیری: 49685355310284)</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4581,7 @@
       </c>
       <c r="L46" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M46" s="13" t="n">
@@ -4580,7 +4600,7 @@
       </c>
       <c r="Q46" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:39 (کد پیگیری: 49685355325246)</t>
         </is>
       </c>
     </row>
@@ -4638,7 +4658,7 @@
       </c>
       <c r="L47" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M47" s="12" t="n">
@@ -4657,7 +4677,7 @@
       </c>
       <c r="Q47" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:14 (کد پیگیری: 49685355340289)</t>
         </is>
       </c>
     </row>
@@ -4715,7 +4735,7 @@
       </c>
       <c r="L48" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>حفظ تاریخچه معتبر قبلی</t>
         </is>
       </c>
       <c r="M48" s="13" t="n">
@@ -4734,7 +4754,7 @@
       </c>
       <c r="Q48" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>عدم حضور در کارتابل امروز؛ حفظ آخرین استعلام معتبر (2026-09-05 08:42:05) (کد پیگیری قبلی: 49682941988821)</t>
         </is>
       </c>
     </row>
@@ -4792,7 +4812,7 @@
       </c>
       <c r="L49" s="7" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M49" s="12" t="n">
@@ -4807,7 +4827,7 @@
       <c r="P49" s="6" t="inlineStr"/>
       <c r="Q49" s="7" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -4880,7 +4900,7 @@
       <c r="P50" s="10" t="inlineStr"/>
       <c r="Q50" s="11" t="inlineStr">
         <is>
-          <t>سررسید چک در تاریخ 1405/06/05 منقضی شده و از کارتابل خارج است</t>
+          <t>سررسید چک در تاریخ 1405/06/05 منقضی شده و از کارتابل جاری خارج است</t>
         </is>
       </c>
     </row>
@@ -4938,7 +4958,7 @@
       </c>
       <c r="L51" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>حفظ تاریخچه معتبر قبلی</t>
         </is>
       </c>
       <c r="M51" s="12" t="n">
@@ -4957,7 +4977,7 @@
       </c>
       <c r="Q51" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>عدم حضور در کارتابل امروز؛ حفظ آخرین استعلام معتبر (2026-09-05 08:46:58) (کد پیگیری قبلی: 49682942078736)</t>
         </is>
       </c>
     </row>
@@ -5015,7 +5035,7 @@
       </c>
       <c r="L52" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M52" s="13" t="n">
@@ -5034,7 +5054,7 @@
       </c>
       <c r="Q52" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:15 (کد پیگیری: 49685355321656)</t>
         </is>
       </c>
     </row>
@@ -5092,7 +5112,7 @@
       </c>
       <c r="L53" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M53" s="12" t="n">
@@ -5111,7 +5131,7 @@
       </c>
       <c r="Q53" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:45 (کد پیگیری: 49685355335056)</t>
         </is>
       </c>
     </row>
@@ -5169,7 +5189,7 @@
       </c>
       <c r="L54" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M54" s="13" t="n">
@@ -5188,7 +5208,7 @@
       </c>
       <c r="Q54" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:24:02 (کد پیگیری: 49685355362164)</t>
         </is>
       </c>
     </row>
@@ -5246,7 +5266,7 @@
       </c>
       <c r="L55" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M55" s="12" t="n">
@@ -5265,7 +5285,7 @@
       </c>
       <c r="Q55" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:20:56 (کد پیگیری: 49685355290024)</t>
         </is>
       </c>
     </row>
@@ -5323,7 +5343,7 @@
       </c>
       <c r="L56" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>حفظ تاریخچه معتبر قبلی</t>
         </is>
       </c>
       <c r="M56" s="13" t="n">
@@ -5342,7 +5362,7 @@
       </c>
       <c r="Q56" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>عدم حضور در کارتابل امروز؛ حفظ آخرین استعلام معتبر (2026-08-28 20:51:57) (کد پیگیری قبلی: 49664982347170)</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5420,7 @@
       </c>
       <c r="L57" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M57" s="12" t="n">
@@ -5419,7 +5439,7 @@
       </c>
       <c r="Q57" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:16 (کد پیگیری: 49685355321681)</t>
         </is>
       </c>
     </row>
@@ -5477,7 +5497,7 @@
       </c>
       <c r="L58" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M58" s="13" t="n">
@@ -5496,7 +5516,7 @@
       </c>
       <c r="Q58" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:44 (کد پیگیری: 49685355345947)</t>
         </is>
       </c>
     </row>
@@ -5569,7 +5589,7 @@
       <c r="P59" s="6" t="inlineStr"/>
       <c r="Q59" s="7" t="inlineStr">
         <is>
-          <t>سررسید چک در تاریخ 1405/06/02 منقضی شده و از کارتابل خارج است</t>
+          <t>سررسید چک در تاریخ 1405/06/02 منقضی شده و از کارتابل جاری خارج است</t>
         </is>
       </c>
     </row>
@@ -5627,7 +5647,7 @@
       </c>
       <c r="L60" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M60" s="13" t="n">
@@ -5646,7 +5666,7 @@
       </c>
       <c r="Q60" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:39 (کد پیگیری: 49685355295883)</t>
         </is>
       </c>
     </row>
@@ -5704,7 +5724,7 @@
       </c>
       <c r="L61" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M61" s="12" t="n">
@@ -5723,7 +5743,7 @@
       </c>
       <c r="Q61" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:13 (کد پیگیری: 49685355317164)</t>
         </is>
       </c>
     </row>
@@ -5781,7 +5801,7 @@
       </c>
       <c r="L62" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M62" s="13" t="n">
@@ -5800,7 +5820,7 @@
       </c>
       <c r="Q62" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:42 (کد پیگیری: 49685355330603)</t>
         </is>
       </c>
     </row>
@@ -5858,7 +5878,7 @@
       </c>
       <c r="L63" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M63" s="12" t="n">
@@ -5877,7 +5897,7 @@
       </c>
       <c r="Q63" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:18 (کد پیگیری: 49685355337378)</t>
         </is>
       </c>
     </row>
@@ -5935,7 +5955,7 @@
       </c>
       <c r="L64" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M64" s="13" t="n">
@@ -5954,7 +5974,7 @@
       </c>
       <c r="Q64" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:36 (کد پیگیری: 49685355342412)</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6032,7 @@
       </c>
       <c r="L65" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M65" s="12" t="n">
@@ -6031,7 +6051,7 @@
       </c>
       <c r="Q65" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:46 (کد پیگیری: 49685355351800)</t>
         </is>
       </c>
     </row>
@@ -6089,7 +6109,7 @@
       </c>
       <c r="L66" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M66" s="13" t="n">
@@ -6108,7 +6128,7 @@
       </c>
       <c r="Q66" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:49 (کد پیگیری: 49685355351842)</t>
         </is>
       </c>
     </row>
@@ -6166,7 +6186,7 @@
       </c>
       <c r="L67" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M67" s="12" t="n">
@@ -6185,7 +6205,7 @@
       </c>
       <c r="Q67" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:50 (کد پیگیری: 49685355359143)</t>
         </is>
       </c>
     </row>
@@ -6243,7 +6263,7 @@
       </c>
       <c r="L68" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M68" s="13" t="n">
@@ -6262,7 +6282,7 @@
       </c>
       <c r="Q68" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:51 (کد پیگیری: 49685355356744)</t>
         </is>
       </c>
     </row>
@@ -6320,7 +6340,7 @@
       </c>
       <c r="L69" s="7" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M69" s="12" t="n">
@@ -6335,7 +6355,7 @@
       <c r="P69" s="6" t="inlineStr"/>
       <c r="Q69" s="7" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6413,7 @@
       </c>
       <c r="L70" s="11" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M70" s="13" t="n">
@@ -6408,7 +6428,7 @@
       <c r="P70" s="10" t="inlineStr"/>
       <c r="Q70" s="11" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -6481,7 +6501,7 @@
       <c r="P71" s="6" t="inlineStr"/>
       <c r="Q71" s="7" t="inlineStr">
         <is>
-          <t>سررسید چک در تاریخ 1405/06/06 منقضی شده و از کارتابل خارج است</t>
+          <t>سررسید چک در تاریخ 1405/06/06 منقضی شده و از کارتابل جاری خارج است</t>
         </is>
       </c>
     </row>
@@ -6539,7 +6559,7 @@
       </c>
       <c r="L72" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M72" s="13" t="n">
@@ -6558,7 +6578,7 @@
       </c>
       <c r="Q72" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:45 (کد پیگیری: 49685355304716)</t>
         </is>
       </c>
     </row>
@@ -6616,7 +6636,7 @@
       </c>
       <c r="L73" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M73" s="12" t="n">
@@ -6635,7 +6655,7 @@
       </c>
       <c r="Q73" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:19 (کد پیگیری: 49685355310375)</t>
         </is>
       </c>
     </row>
@@ -6693,7 +6713,7 @@
       </c>
       <c r="L74" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M74" s="13" t="n">
@@ -6712,7 +6732,7 @@
       </c>
       <c r="Q74" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:23 (کد پیگیری: 49685355339937)</t>
         </is>
       </c>
     </row>
@@ -6766,7 +6786,7 @@
       </c>
       <c r="L75" s="7" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M75" s="12" t="n">
@@ -6781,7 +6801,7 @@
       <c r="P75" s="6" t="inlineStr"/>
       <c r="Q75" s="7" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -6900,7 +6920,7 @@
       </c>
       <c r="L77" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M77" s="12" t="n">
@@ -6919,7 +6939,7 @@
       </c>
       <c r="Q77" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:41 (کد پیگیری: 49685355328166)</t>
         </is>
       </c>
     </row>
@@ -6988,7 +7008,7 @@
       <c r="P78" s="10" t="inlineStr"/>
       <c r="Q78" s="11" t="inlineStr">
         <is>
-          <t>سررسید چک در تاریخ 1405/06/05 منقضی شده و از کارتابل خارج است</t>
+          <t>سررسید چک در تاریخ 1405/06/05 منقضی شده و از کارتابل جاری خارج است</t>
         </is>
       </c>
     </row>
@@ -7046,7 +7066,7 @@
       </c>
       <c r="L79" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>حفظ تاریخچه معتبر قبلی</t>
         </is>
       </c>
       <c r="M79" s="12" t="n">
@@ -7065,7 +7085,7 @@
       </c>
       <c r="Q79" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>عدم حضور در کارتابل امروز؛ حفظ آخرین استعلام معتبر (2026-09-05 08:46:41) (کد پیگیری قبلی: 49682942080036)</t>
         </is>
       </c>
     </row>
@@ -7123,7 +7143,7 @@
       </c>
       <c r="L80" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M80" s="13" t="n">
@@ -7142,7 +7162,7 @@
       </c>
       <c r="Q80" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:55 (کد پیگیری: 49685355305280)</t>
         </is>
       </c>
     </row>
@@ -7200,7 +7220,7 @@
       </c>
       <c r="L81" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M81" s="12" t="n">
@@ -7219,7 +7239,7 @@
       </c>
       <c r="Q81" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:27 (کد پیگیری: 49685355323218)</t>
         </is>
       </c>
     </row>
@@ -7277,7 +7297,7 @@
       </c>
       <c r="L82" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M82" s="13" t="n">
@@ -7296,7 +7316,7 @@
       </c>
       <c r="Q82" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:00 (کد پیگیری: 49685355327928)</t>
         </is>
       </c>
     </row>
@@ -7354,7 +7374,7 @@
       </c>
       <c r="L83" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M83" s="12" t="n">
@@ -7373,7 +7393,7 @@
       </c>
       <c r="Q83" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:27 (کد پیگیری: 49685355351557)</t>
         </is>
       </c>
     </row>
@@ -7431,7 +7451,7 @@
       </c>
       <c r="L84" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M84" s="13" t="n">
@@ -7450,7 +7470,7 @@
       </c>
       <c r="Q84" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:00 (کد پیگیری: 49685355305344)</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7528,7 @@
       </c>
       <c r="L85" s="7" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M85" s="12" t="n">
@@ -7523,7 +7543,7 @@
       <c r="P85" s="6" t="inlineStr"/>
       <c r="Q85" s="7" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -7581,7 +7601,7 @@
       </c>
       <c r="L86" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M86" s="13" t="n">
@@ -7600,7 +7620,7 @@
       </c>
       <c r="Q86" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:59 (کد پیگیری: 49685355307268)</t>
         </is>
       </c>
     </row>
@@ -7658,7 +7678,7 @@
       </c>
       <c r="L87" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M87" s="12" t="n">
@@ -7677,7 +7697,7 @@
       </c>
       <c r="Q87" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:18 (کد پیگیری: 49685355297097)</t>
         </is>
       </c>
     </row>
@@ -7735,7 +7755,7 @@
       </c>
       <c r="L88" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M88" s="13" t="n">
@@ -7754,7 +7774,7 @@
       </c>
       <c r="Q88" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:30 (کد پیگیری: 49685355323269)</t>
         </is>
       </c>
     </row>
@@ -7812,7 +7832,7 @@
       </c>
       <c r="L89" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M89" s="12" t="n">
@@ -7831,7 +7851,7 @@
       </c>
       <c r="Q89" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:20:54 (کد پیگیری: 49685355273867)</t>
         </is>
       </c>
     </row>
@@ -7889,7 +7909,7 @@
       </c>
       <c r="L90" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M90" s="13" t="n">
@@ -7908,7 +7928,7 @@
       </c>
       <c r="Q90" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:20:58 (کد پیگیری: 49685355276364)</t>
         </is>
       </c>
     </row>
@@ -7966,7 +7986,7 @@
       </c>
       <c r="L91" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M91" s="12" t="n">
@@ -7985,7 +8005,7 @@
       </c>
       <c r="Q91" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:10 (کد پیگیری: 49685355321584)</t>
         </is>
       </c>
     </row>
@@ -8043,7 +8063,7 @@
       </c>
       <c r="L92" s="11" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M92" s="13" t="n">
@@ -8058,7 +8078,7 @@
       <c r="P92" s="10" t="inlineStr"/>
       <c r="Q92" s="11" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -8116,7 +8136,7 @@
       </c>
       <c r="L93" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M93" s="12" t="n">
@@ -8135,7 +8155,7 @@
       </c>
       <c r="Q93" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:38 (کد پیگیری: 49685355330069)</t>
         </is>
       </c>
     </row>
@@ -8193,7 +8213,7 @@
       </c>
       <c r="L94" s="11" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M94" s="13" t="n">
@@ -8208,7 +8228,7 @@
       <c r="P94" s="10" t="inlineStr"/>
       <c r="Q94" s="11" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -8266,7 +8286,7 @@
       </c>
       <c r="L95" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M95" s="12" t="n">
@@ -8285,7 +8305,7 @@
       </c>
       <c r="Q95" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:12 (کد پیگیری: 49685355338321)</t>
         </is>
       </c>
     </row>
@@ -8343,7 +8363,7 @@
       </c>
       <c r="L96" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M96" s="13" t="n">
@@ -8362,7 +8382,7 @@
       </c>
       <c r="Q96" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:33 (کد پیگیری: 49685355355077)</t>
         </is>
       </c>
     </row>
@@ -8431,7 +8451,7 @@
       <c r="P97" s="6" t="inlineStr"/>
       <c r="Q97" s="7" t="inlineStr">
         <is>
-          <t>سررسید چک در تاریخ 1405/06/01 منقضی شده و از کارتابل خارج است</t>
+          <t>سررسید چک در تاریخ 1405/06/01 منقضی شده و از کارتابل جاری خارج است</t>
         </is>
       </c>
     </row>
@@ -8489,7 +8509,7 @@
       </c>
       <c r="L98" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M98" s="13" t="n">
@@ -8508,7 +8528,7 @@
       </c>
       <c r="Q98" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:24 (کد پیگیری: 49685355289857)</t>
         </is>
       </c>
     </row>
@@ -8566,7 +8586,7 @@
       </c>
       <c r="L99" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>حفظ تاریخچه معتبر قبلی</t>
         </is>
       </c>
       <c r="M99" s="12" t="n">
@@ -8585,7 +8605,7 @@
       </c>
       <c r="Q99" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>عدم حضور در کارتابل امروز؛ حفظ آخرین استعلام معتبر (2026-09-05 08:45:48) (کد پیگیری قبلی: 49682942065011)</t>
         </is>
       </c>
     </row>
@@ -8643,7 +8663,7 @@
       </c>
       <c r="L100" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M100" s="13" t="n">
@@ -8662,7 +8682,7 @@
       </c>
       <c r="Q100" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:04 (کد پیگیری: 49685355310220)</t>
         </is>
       </c>
     </row>
@@ -8720,7 +8740,7 @@
       </c>
       <c r="L101" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M101" s="12" t="n">
@@ -8739,7 +8759,7 @@
       </c>
       <c r="Q101" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:33 (کد پیگیری: 49685355326605)</t>
         </is>
       </c>
     </row>
@@ -8797,7 +8817,7 @@
       </c>
       <c r="L102" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M102" s="13" t="n">
@@ -8816,7 +8836,7 @@
       </c>
       <c r="Q102" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:55 (کد پیگیری: 49685355356775)</t>
         </is>
       </c>
     </row>
@@ -8874,7 +8894,7 @@
       </c>
       <c r="L103" s="7" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M103" s="12" t="n">
@@ -8889,7 +8909,7 @@
       <c r="P103" s="6" t="inlineStr"/>
       <c r="Q103" s="7" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -8947,7 +8967,7 @@
       </c>
       <c r="L104" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>حفظ تاریخچه معتبر قبلی</t>
         </is>
       </c>
       <c r="M104" s="13" t="n">
@@ -8966,7 +8986,7 @@
       </c>
       <c r="Q104" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>عدم حضور در کارتابل امروز؛ حفظ آخرین استعلام معتبر (2026-09-05 08:47:08) (کد پیگیری قبلی: 49682942084694)</t>
         </is>
       </c>
     </row>
@@ -9024,7 +9044,7 @@
       </c>
       <c r="L105" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M105" s="12" t="n">
@@ -9043,7 +9063,7 @@
       </c>
       <c r="Q105" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:24 (کد پیگیری: 49685355318270)</t>
         </is>
       </c>
     </row>
@@ -9116,7 +9136,7 @@
       <c r="P106" s="10" t="inlineStr"/>
       <c r="Q106" s="11" t="inlineStr">
         <is>
-          <t>سررسید چک در تاریخ 1405/06/11 منقضی شده و از کارتابل خارج است</t>
+          <t>سررسید چک در تاریخ 1405/06/11 منقضی شده و از کارتابل جاری خارج است</t>
         </is>
       </c>
     </row>
@@ -9174,7 +9194,7 @@
       </c>
       <c r="L107" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M107" s="12" t="n">
@@ -9193,7 +9213,7 @@
       </c>
       <c r="Q107" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:44 (کد پیگیری: 49685355330620)</t>
         </is>
       </c>
     </row>
@@ -9251,7 +9271,7 @@
       </c>
       <c r="L108" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M108" s="13" t="n">
@@ -9270,7 +9290,7 @@
       </c>
       <c r="Q108" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:51 (کد پیگیری: 49685355327817)</t>
         </is>
       </c>
     </row>
@@ -9328,7 +9348,7 @@
       </c>
       <c r="L109" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M109" s="12" t="n">
@@ -9347,7 +9367,7 @@
       </c>
       <c r="Q109" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:56 (کد پیگیری: 49685355336594)</t>
         </is>
       </c>
     </row>
@@ -9405,7 +9425,7 @@
       </c>
       <c r="L110" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M110" s="13" t="n">
@@ -9424,7 +9444,7 @@
       </c>
       <c r="Q110" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:58 (کد پیگیری: 49685355335702)</t>
         </is>
       </c>
     </row>
@@ -9482,7 +9502,7 @@
       </c>
       <c r="L111" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M111" s="12" t="n">
@@ -9501,7 +9521,7 @@
       </c>
       <c r="Q111" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:02 (کد پیگیری: 49685355327942)</t>
         </is>
       </c>
     </row>
@@ -9559,7 +9579,7 @@
       </c>
       <c r="L112" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M112" s="13" t="n">
@@ -9578,7 +9598,7 @@
       </c>
       <c r="Q112" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:09 (کد پیگیری: 49685355345013)</t>
         </is>
       </c>
     </row>
@@ -9636,7 +9656,7 @@
       </c>
       <c r="L113" s="7" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M113" s="12" t="n">
@@ -9651,7 +9671,7 @@
       <c r="P113" s="6" t="inlineStr"/>
       <c r="Q113" s="7" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -9724,7 +9744,7 @@
       <c r="P114" s="10" t="inlineStr"/>
       <c r="Q114" s="11" t="inlineStr">
         <is>
-          <t>سررسید چک در تاریخ 1405/06/01 منقضی شده و از کارتابل خارج است</t>
+          <t>سررسید چک در تاریخ 1405/06/01 منقضی شده و از کارتابل جاری خارج است</t>
         </is>
       </c>
     </row>
@@ -9782,7 +9802,7 @@
       </c>
       <c r="L115" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M115" s="12" t="n">
@@ -9801,7 +9821,7 @@
       </c>
       <c r="Q115" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:36 (کد پیگیری: 49685355299734)</t>
         </is>
       </c>
     </row>
@@ -9859,7 +9879,7 @@
       </c>
       <c r="L116" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>حفظ تاریخچه معتبر قبلی</t>
         </is>
       </c>
       <c r="M116" s="13" t="n">
@@ -9878,7 +9898,7 @@
       </c>
       <c r="Q116" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>عدم حضور در کارتابل امروز؛ حفظ آخرین استعلام معتبر (2026-08-28 20:53:55) (کد پیگیری قبلی: 49664982349765)</t>
         </is>
       </c>
     </row>
@@ -9936,7 +9956,7 @@
       </c>
       <c r="L117" s="7" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M117" s="12" t="n">
@@ -9951,7 +9971,7 @@
       <c r="P117" s="6" t="inlineStr"/>
       <c r="Q117" s="7" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -10009,7 +10029,7 @@
       </c>
       <c r="L118" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M118" s="13" t="n">
@@ -10028,7 +10048,7 @@
       </c>
       <c r="Q118" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:17 (کد پیگیری: 49685355338378)</t>
         </is>
       </c>
     </row>
@@ -10086,7 +10106,7 @@
       </c>
       <c r="L119" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M119" s="12" t="n">
@@ -10105,7 +10125,7 @@
       </c>
       <c r="Q119" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:35 (کد پیگیری: 49685355346272)</t>
         </is>
       </c>
     </row>
@@ -10163,7 +10183,7 @@
       </c>
       <c r="L120" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M120" s="13" t="n">
@@ -10182,7 +10202,7 @@
       </c>
       <c r="Q120" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:54 (کد پیگیری: 49685355356761)</t>
         </is>
       </c>
     </row>
@@ -10240,7 +10260,7 @@
       </c>
       <c r="L121" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M121" s="12" t="n">
@@ -10259,7 +10279,7 @@
       </c>
       <c r="Q121" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:57 (کد پیگیری: 49685355362576)</t>
         </is>
       </c>
     </row>
@@ -10317,7 +10337,7 @@
       </c>
       <c r="L122" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M122" s="13" t="n">
@@ -10336,7 +10356,7 @@
       </c>
       <c r="Q122" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:24:00 (کد پیگیری: 49685355359253)</t>
         </is>
       </c>
     </row>
@@ -10394,7 +10414,7 @@
       </c>
       <c r="L123" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M123" s="12" t="n">
@@ -10413,7 +10433,7 @@
       </c>
       <c r="Q123" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:03 (کد پیگیری: 49685355304941)</t>
         </is>
       </c>
     </row>
@@ -10471,7 +10491,7 @@
       </c>
       <c r="L124" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M124" s="13" t="n">
@@ -10490,7 +10510,7 @@
       </c>
       <c r="Q124" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:29 (کد پیگیری: 49685355323252)</t>
         </is>
       </c>
     </row>
@@ -10548,7 +10568,7 @@
       </c>
       <c r="L125" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M125" s="12" t="n">
@@ -10567,7 +10587,7 @@
       </c>
       <c r="Q125" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:05 (کد پیگیری: 49685355336252)</t>
         </is>
       </c>
     </row>
@@ -10625,7 +10645,7 @@
       </c>
       <c r="L126" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M126" s="13" t="n">
@@ -10644,7 +10664,7 @@
       </c>
       <c r="Q126" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:13 (کد پیگیری: 49685355332442)</t>
         </is>
       </c>
     </row>
@@ -10702,7 +10722,7 @@
       </c>
       <c r="L127" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M127" s="12" t="n">
@@ -10721,7 +10741,7 @@
       </c>
       <c r="Q127" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:30 (کد پیگیری: 49685355351603)</t>
         </is>
       </c>
     </row>
@@ -10779,7 +10799,7 @@
       </c>
       <c r="L128" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M128" s="13" t="n">
@@ -10798,7 +10818,7 @@
       </c>
       <c r="Q128" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:41 (کد پیگیری: 49685355348870)</t>
         </is>
       </c>
     </row>
@@ -10856,7 +10876,7 @@
       </c>
       <c r="L129" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M129" s="12" t="n">
@@ -10875,7 +10895,7 @@
       </c>
       <c r="Q129" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:45 (کد پیگیری: 49685355345963)</t>
         </is>
       </c>
     </row>
@@ -10933,7 +10953,7 @@
       </c>
       <c r="L130" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M130" s="13" t="n">
@@ -10952,7 +10972,7 @@
       </c>
       <c r="Q130" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:06 (کد پیگیری: 49685355308315)</t>
         </is>
       </c>
     </row>
@@ -11010,7 +11030,7 @@
       </c>
       <c r="L131" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M131" s="12" t="n">
@@ -11029,7 +11049,7 @@
       </c>
       <c r="Q131" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:56 (کد پیگیری: 49685355307242)</t>
         </is>
       </c>
     </row>
@@ -11087,7 +11107,7 @@
       </c>
       <c r="L132" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M132" s="13" t="n">
@@ -11106,7 +11126,7 @@
       </c>
       <c r="Q132" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:20 (کد پیگیری: 49685355297107)</t>
         </is>
       </c>
     </row>
@@ -11164,7 +11184,7 @@
       </c>
       <c r="L133" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M133" s="12" t="n">
@@ -11183,7 +11203,7 @@
       </c>
       <c r="Q133" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:29 (کد پیگیری: 49685355303545)</t>
         </is>
       </c>
     </row>
@@ -11241,7 +11261,7 @@
       </c>
       <c r="L134" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>حفظ تاریخچه معتبر قبلی</t>
         </is>
       </c>
       <c r="M134" s="13" t="n">
@@ -11260,7 +11280,7 @@
       </c>
       <c r="Q134" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>عدم حضور در کارتابل امروز؛ حفظ آخرین استعلام معتبر (2026-09-05 08:47:12) (کد پیگیری قبلی: 49682942089573)</t>
         </is>
       </c>
     </row>
@@ -11318,7 +11338,7 @@
       </c>
       <c r="L135" s="7" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M135" s="12" t="n">
@@ -11333,7 +11353,7 @@
       <c r="P135" s="6" t="inlineStr"/>
       <c r="Q135" s="7" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -11391,7 +11411,7 @@
       </c>
       <c r="L136" s="11" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M136" s="13" t="n">
@@ -11406,7 +11426,7 @@
       <c r="P136" s="10" t="inlineStr"/>
       <c r="Q136" s="11" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -11464,7 +11484,7 @@
       </c>
       <c r="L137" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M137" s="12" t="n">
@@ -11483,7 +11503,7 @@
       </c>
       <c r="Q137" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:07 (کد پیگیری: 49685355318094)</t>
         </is>
       </c>
     </row>
@@ -11541,7 +11561,7 @@
       </c>
       <c r="L138" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M138" s="13" t="n">
@@ -11560,7 +11580,7 @@
       </c>
       <c r="Q138" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:06 (کد پیگیری: 49685355344022)</t>
         </is>
       </c>
     </row>
@@ -11618,7 +11638,7 @@
       </c>
       <c r="L139" s="7" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M139" s="12" t="n">
@@ -11633,7 +11653,7 @@
       <c r="P139" s="6" t="inlineStr"/>
       <c r="Q139" s="7" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -11691,7 +11711,7 @@
       </c>
       <c r="L140" s="11" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M140" s="13" t="n">
@@ -11706,7 +11726,7 @@
       <c r="P140" s="10" t="inlineStr"/>
       <c r="Q140" s="11" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -11764,7 +11784,7 @@
       </c>
       <c r="L141" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M141" s="12" t="n">
@@ -11783,7 +11803,7 @@
       </c>
       <c r="Q141" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:57 (کد پیگیری: 49685355304887)</t>
         </is>
       </c>
     </row>
@@ -11841,7 +11861,7 @@
       </c>
       <c r="L142" s="11" t="inlineStr">
         <is>
-          <t>حفظ تاریخچه معتبر</t>
+          <t>عدم حضور در کارتابل ۹ دارنده</t>
         </is>
       </c>
       <c r="M142" s="13" t="n">
@@ -11856,7 +11876,7 @@
       <c r="P142" s="10" t="inlineStr"/>
       <c r="Q142" s="11" t="inlineStr">
         <is>
-          <t>اطلاعات معتبر آخرین استعلام موفق حفظ شد</t>
+          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
         </is>
       </c>
     </row>
@@ -11914,7 +11934,7 @@
       </c>
       <c r="L143" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M143" s="12" t="n">
@@ -11933,7 +11953,7 @@
       </c>
       <c r="Q143" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:22:28 (کد پیگیری: 49685355318322)</t>
         </is>
       </c>
     </row>
@@ -11991,7 +12011,7 @@
       </c>
       <c r="L144" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M144" s="13" t="n">
@@ -12010,7 +12030,7 @@
       </c>
       <c r="Q144" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:23:28 (کد پیگیری: 49685355346211)</t>
         </is>
       </c>
     </row>
@@ -12068,7 +12088,7 @@
       </c>
       <c r="L145" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M145" s="12" t="n">
@@ -12087,7 +12107,7 @@
       </c>
       <c r="Q145" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:13 (کد پیگیری: 49685355294555)</t>
         </is>
       </c>
     </row>
@@ -12145,7 +12165,7 @@
       </c>
       <c r="L146" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M146" s="13" t="n">
@@ -12164,7 +12184,7 @@
       </c>
       <c r="Q146" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:31 (کد پیگیری: 49685355291850)</t>
         </is>
       </c>
     </row>
@@ -12222,7 +12242,7 @@
       </c>
       <c r="L147" s="7" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M147" s="12" t="n">
@@ -12241,7 +12261,7 @@
       </c>
       <c r="Q147" s="7" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:09 (کد پیگیری: 49685355289191)</t>
         </is>
       </c>
     </row>
@@ -12299,7 +12319,7 @@
       </c>
       <c r="L148" s="11" t="inlineStr">
         <is>
-          <t>موفق (درگاه زنده)</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M148" s="13" t="n">
@@ -12318,7 +12338,7 @@
       </c>
       <c r="Q148" s="11" t="inlineStr">
         <is>
-          <t>استعلام زنده از درگاه پاسارگاد با موفقیت ثبت شد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 09:21:49 (کد پیگیری: 49685355309095)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(pasargad): fix cascade logic skipping holders 2-9, sync Zahra Bahrami red credit color and bounced inquiry
</commit_message>
<xml_diff>
--- a/گزارش_جامع_استعلام_چک_ها_۱۴۰۵۰۶۱۵.xlsx
+++ b/گزارش_جامع_استعلام_چک_ها_۱۴۰۵۰۶۱۵.xlsx
@@ -635,7 +635,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>سامانه صیاد پرو ۳.۱ | تاریخ تهیه گزارش: 1405/06/15 ساعت 16:05:36 | منبع داده: درگاه رسمی بانک مرکزی و بانک پاسارگاد</t>
+          <t>سامانه صیاد پرو ۳.۱ | تاریخ تهیه گزارش: 1405/06/15 ساعت 18:54:36 | منبع داده: درگاه رسمی بانک مرکزی و بانک پاسارگاد</t>
         </is>
       </c>
     </row>
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>16109551207163</v>
+        <v>16448381207163</v>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
@@ -738,7 +738,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>1,610,955 تومان (تعهدات صادرکنندگان در شبکه بانکی)</t>
+          <t>1,644,838 تومان (تعهدات صادرکنندگان در شبکه بانکی)</t>
         </is>
       </c>
     </row>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>4064396530614</v>
+        <v>4076196530614</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
@@ -758,7 +758,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>406,440 تومان (سابقه تسویه موفق)</t>
+          <t>407,620 تومان (سابقه تسویه موفق)</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>589878000000</v>
+        <v>602178000000</v>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>58,988 تومان (چک‌های برگشتی ثبت‌شده بانک مرکزی)</t>
+          <t>60,218 تومان (چک‌های برگشتی ثبت‌شده بانک مرکزی)</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
@@ -919,10 +919,10 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C19" s="16" t="n">
-        <v>0.6923076923076923</v>
+        <v>0.6730769230769231</v>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
@@ -937,10 +937,10 @@
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C20" s="17" t="n">
-        <v>0.2692307692307692</v>
+        <v>0.2884615384615384</v>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
@@ -1003,10 +1003,10 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C25" s="12" t="n">
-        <v>305440000000</v>
+        <v>290440000000</v>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
@@ -1057,10 +1057,10 @@
         </is>
       </c>
       <c r="B28" s="9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C28" s="13" t="n">
-        <v>134700000000</v>
+        <v>149700000000</v>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
@@ -3632,10 +3632,14 @@
           <t>زهرا بهرامي پويا</t>
         </is>
       </c>
-      <c r="C34" s="10" t="inlineStr"/>
-      <c r="D34" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>0927624011</t>
+        </is>
+      </c>
+      <c r="D34" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E34" s="10" t="inlineStr">
@@ -3668,27 +3672,31 @@
       </c>
       <c r="K34" s="11" t="inlineStr">
         <is>
-          <t>علی رمضانزاده</t>
+          <t>فاطمه زمانزاده</t>
         </is>
       </c>
       <c r="L34" s="11" t="inlineStr">
         <is>
-          <t>عدم حضور در کارتابل ۹ دارنده</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M34" s="13" t="n">
-        <v>0</v>
+        <v>338830000000</v>
       </c>
       <c r="N34" s="13" t="n">
-        <v>0</v>
+        <v>11800000000</v>
       </c>
       <c r="O34" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P34" s="10" t="inlineStr"/>
+        <v>12300000000</v>
+      </c>
+      <c r="P34" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-06 18:54:14</t>
+        </is>
+      </c>
       <c r="Q34" s="11" t="inlineStr">
         <is>
-          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 18:54:14 (کد پیگیری: 49686363251893)</t>
         </is>
       </c>
     </row>
@@ -13265,23 +13273,27 @@
           <t>زهرا بهرامي پويا</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr"/>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>0927624011</t>
+        </is>
+      </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>سفید</t>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E18" s="10" t="n">
-        <v>87</v>
-      </c>
-      <c r="F18" s="24" t="inlineStr">
-        <is>
-          <t>عالی</t>
+        <v>0</v>
+      </c>
+      <c r="F18" s="23" t="inlineStr">
+        <is>
+          <t>پرخطر</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>کم‌ریسک و پرتراکنش (ستاره‌ها و مشتریان طلایی)</t>
+          <t>پرریسک با تعهدات سنگین (هشدار قرمز و بحرانی)</t>
         </is>
       </c>
       <c r="H18" s="10" t="n">
@@ -13291,14 +13303,14 @@
         <v>15000000000</v>
       </c>
       <c r="J18" s="13" t="n">
-        <v>0</v>
+        <v>338830000000</v>
       </c>
       <c r="K18" s="13" t="n">
-        <v>0</v>
+        <v>12300000000</v>
       </c>
       <c r="L18" s="11" t="inlineStr">
         <is>
-          <t>مشتری ممتاز با سلامت مالی درخشان. واجد شرایط دریافت بالاترین سقف اعتبار و تسهیلات تجاری.</t>
+          <t>هشدار بحرانی: سلامت مالی بسیار ضعیف و احتمال بالای نکول. از پذیرش هرگونه چک جدید اکیداً خودداری شود.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(customers): audit and sync all 5 bounced customers to RED credit color and regenerate excel
</commit_message>
<xml_diff>
--- a/گزارش_جامع_استعلام_چک_ها_۱۴۰۵۰۶۱۵.xlsx
+++ b/گزارش_جامع_استعلام_چک_ها_۱۴۰۵۰۶۱۵.xlsx
@@ -635,7 +635,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>سامانه صیاد پرو ۳.۱ | تاریخ تهیه گزارش: 1405/06/15 ساعت 18:54:36 | منبع داده: درگاه رسمی بانک مرکزی و بانک پاسارگاد</t>
+          <t>سامانه صیاد پرو ۳.۱ | تاریخ تهیه گزارش: 1405/06/15 ساعت 19:02:20 | منبع داده: درگاه رسمی بانک مرکزی و بانک پاسارگاد</t>
         </is>
       </c>
     </row>
@@ -919,10 +919,10 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C19" s="16" t="n">
-        <v>0.6730769230769231</v>
+        <v>0.6153846153846154</v>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
@@ -937,10 +937,10 @@
         </is>
       </c>
       <c r="B20" s="9" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C20" s="17" t="n">
-        <v>0.2884615384615384</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
@@ -955,10 +955,10 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C21" s="16" t="n">
-        <v>0.03846153846153846</v>
+        <v>0</v>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
@@ -1003,10 +1003,10 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C25" s="12" t="n">
-        <v>290440000000</v>
+        <v>235690000000</v>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
@@ -1057,10 +1057,10 @@
         </is>
       </c>
       <c r="B28" s="9" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C28" s="13" t="n">
-        <v>149700000000</v>
+        <v>204450000000</v>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
@@ -2336,9 +2336,9 @@
           <t>0941314121</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>قهوه ای</t>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
@@ -2413,9 +2413,9 @@
           <t>0941314121</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>قهوه ای</t>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E18" s="10" t="inlineStr">
@@ -2490,9 +2490,9 @@
           <t>0941314121</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>قهوه ای</t>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -2567,9 +2567,9 @@
           <t>0941314121</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>قهوه ای</t>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
@@ -2644,9 +2644,9 @@
           <t>0941314121</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>قهوه ای</t>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
@@ -2721,9 +2721,9 @@
           <t>0941314121</t>
         </is>
       </c>
-      <c r="D22" s="11" t="inlineStr">
-        <is>
-          <t>قهوه ای</t>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
@@ -2798,9 +2798,9 @@
           <t>0941314121</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>قهوه ای</t>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
@@ -5234,9 +5234,9 @@
           <t>0922030936</t>
         </is>
       </c>
-      <c r="D55" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D55" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E55" s="6" t="inlineStr">
@@ -5311,9 +5311,9 @@
           <t>0922030936</t>
         </is>
       </c>
-      <c r="D56" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D56" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E56" s="10" t="inlineStr">
@@ -5388,9 +5388,9 @@
           <t>0922030936</t>
         </is>
       </c>
-      <c r="D57" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D57" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr">
@@ -5465,9 +5465,9 @@
           <t>0922030936</t>
         </is>
       </c>
-      <c r="D58" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D58" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E58" s="10" t="inlineStr">
@@ -8477,9 +8477,9 @@
           <t>0922010536</t>
         </is>
       </c>
-      <c r="D98" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D98" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E98" s="10" t="inlineStr">
@@ -8554,9 +8554,9 @@
           <t>0922010536</t>
         </is>
       </c>
-      <c r="D99" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D99" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E99" s="6" t="inlineStr">
@@ -8631,9 +8631,9 @@
           <t>0922010536</t>
         </is>
       </c>
-      <c r="D100" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D100" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E100" s="10" t="inlineStr">
@@ -8708,9 +8708,9 @@
           <t>0922010536</t>
         </is>
       </c>
-      <c r="D101" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D101" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E101" s="6" t="inlineStr">
@@ -8785,9 +8785,9 @@
           <t>0922010536</t>
         </is>
       </c>
-      <c r="D102" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D102" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E102" s="10" t="inlineStr">
@@ -8862,9 +8862,9 @@
           <t>0922010536</t>
         </is>
       </c>
-      <c r="D103" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D103" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E103" s="6" t="inlineStr">
@@ -9089,9 +9089,9 @@
           <t>6430003159</t>
         </is>
       </c>
-      <c r="D106" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D106" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E106" s="10" t="inlineStr">
@@ -9162,9 +9162,9 @@
           <t>6430003159</t>
         </is>
       </c>
-      <c r="D107" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D107" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E107" s="6" t="inlineStr">
@@ -9239,9 +9239,9 @@
           <t>6430003159</t>
         </is>
       </c>
-      <c r="D108" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D108" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E108" s="10" t="inlineStr">
@@ -9316,9 +9316,9 @@
           <t>6430003159</t>
         </is>
       </c>
-      <c r="D109" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D109" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E109" s="6" t="inlineStr">
@@ -9393,9 +9393,9 @@
           <t>6430003159</t>
         </is>
       </c>
-      <c r="D110" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D110" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E110" s="10" t="inlineStr">
@@ -9470,9 +9470,9 @@
           <t>6430003159</t>
         </is>
       </c>
-      <c r="D111" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D111" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E111" s="6" t="inlineStr">
@@ -9547,9 +9547,9 @@
           <t>6430003159</t>
         </is>
       </c>
-      <c r="D112" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D112" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E112" s="10" t="inlineStr">
@@ -9624,9 +9624,9 @@
           <t>6430003159</t>
         </is>
       </c>
-      <c r="D113" s="19" t="inlineStr">
-        <is>
-          <t>سفید</t>
+      <c r="D113" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E113" s="6" t="inlineStr">
@@ -12210,9 +12210,9 @@
           <t>1920394974</t>
         </is>
       </c>
-      <c r="D147" s="7" t="inlineStr">
-        <is>
-          <t>قهوه ای</t>
+      <c r="D147" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E147" s="6" t="inlineStr">
@@ -12287,9 +12287,9 @@
           <t>1920394974</t>
         </is>
       </c>
-      <c r="D148" s="11" t="inlineStr">
-        <is>
-          <t>قهوه ای</t>
+      <c r="D148" s="18" t="inlineStr">
+        <is>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E148" s="10" t="inlineStr">
@@ -12934,11 +12934,11 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>قهوه ای</t>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E11" s="6" t="n">
-        <v>48.8</v>
+        <v>42.8</v>
       </c>
       <c r="F11" s="23" t="inlineStr">
         <is>
@@ -13676,20 +13676,20 @@
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>سفید</t>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E26" s="10" t="n">
-        <v>70</v>
-      </c>
-      <c r="F26" s="24" t="inlineStr">
-        <is>
-          <t>خوب</t>
+        <v>16</v>
+      </c>
+      <c r="F26" s="23" t="inlineStr">
+        <is>
+          <t>پرخطر</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
         <is>
-          <t>کم‌ریسک و پرتراکنش (ستاره‌ها و مشتریان طلایی)</t>
+          <t>پرریسک با تعهدات سنگین (هشدار قرمز و بحرانی)</t>
         </is>
       </c>
       <c r="H26" s="10" t="n">
@@ -13706,7 +13706,7 @@
       </c>
       <c r="L26" s="11" t="inlineStr">
         <is>
-          <t>سلامت مالی مطلوب و کم‌ریسک. تداوم همکاری با رعایت دوره‌های معمول تسویه حساب توصیه می‌شود.</t>
+          <t>هشدار بحرانی: سلامت مالی بسیار ضعیف و احتمال بالای نکول. از پذیرش هرگونه چک جدید اکیداً خودداری شود.</t>
         </is>
       </c>
     </row>
@@ -14310,20 +14310,20 @@
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>سفید</t>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E39" s="6" t="n">
-        <v>79</v>
-      </c>
-      <c r="F39" s="24" t="inlineStr">
-        <is>
-          <t>خوب</t>
+        <v>25</v>
+      </c>
+      <c r="F39" s="23" t="inlineStr">
+        <is>
+          <t>پرخطر</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>کم‌ریسک و پرتراکنش (ستاره‌ها و مشتریان طلایی)</t>
+          <t>پرریسک با تعهدات سنگین (هشدار قرمز و بحرانی)</t>
         </is>
       </c>
       <c r="H39" s="6" t="n">
@@ -14340,7 +14340,7 @@
       </c>
       <c r="L39" s="7" t="inlineStr">
         <is>
-          <t>سلامت مالی مطلوب و کم‌ریسک. تداوم همکاری با رعایت دوره‌های معمول تسویه حساب توصیه می‌شود.</t>
+          <t>هشدار بحرانی: سلامت مالی بسیار ضعیف و احتمال بالای نکول. از پذیرش هرگونه چک جدید اکیداً خودداری شود.</t>
         </is>
       </c>
     </row>
@@ -14410,11 +14410,11 @@
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>سفید</t>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E41" s="6" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="F41" s="23" t="inlineStr">
         <is>
@@ -15010,7 +15010,7 @@
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>قهوه ای</t>
+          <t>قرمز</t>
         </is>
       </c>
       <c r="E53" s="6" t="n">

</xml_diff>

<commit_message>
feat(audit): audit all holders, discover 6 additional cheques on holders 4 & 5, and generate version 3 Excel
</commit_message>
<xml_diff>
--- a/گزارش_جامع_استعلام_چک_ها_۱۴۰۵۰۶۱۵.xlsx
+++ b/گزارش_جامع_استعلام_چک_ها_۱۴۰۵۰۶۱۵.xlsx
@@ -635,7 +635,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>سامانه صیاد پرو ۳.۱ | تاریخ تهیه گزارش: 1405/06/15 ساعت 19:02:20 | منبع داده: درگاه رسمی بانک مرکزی و بانک پاسارگاد</t>
+          <t>سامانه صیاد پرو ۳.۱ | تاریخ تهیه گزارش: 1405/06/15 ساعت 19:14:20 | منبع داده: درگاه رسمی بانک مرکزی و بانک پاسارگاد</t>
         </is>
       </c>
     </row>
@@ -729,7 +729,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>16448381207163</v>
+        <v>16795489807163</v>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
@@ -738,7 +738,7 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>1,644,838 تومان (تعهدات صادرکنندگان در شبکه بانکی)</t>
+          <t>1,679,549 تومان (تعهدات صادرکنندگان در شبکه بانکی)</t>
         </is>
       </c>
     </row>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>4076196530614</v>
+        <v>4117195410614</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
@@ -758,7 +758,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>407,620 تومان (سابقه تسویه موفق)</t>
+          <t>411,720 تومان (سابقه تسویه موفق)</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>602178000000</v>
+        <v>604830000000</v>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>60,218 تومان (چک‌های برگشتی ثبت‌شده بانک مرکزی)</t>
+          <t>60,483 تومان (چک‌های برگشتی ثبت‌شده بانک مرکزی)</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
@@ -4207,27 +4207,31 @@
       </c>
       <c r="K41" s="7" t="inlineStr">
         <is>
-          <t>علی رمضانزاده</t>
+          <t>مهدی زمانزاده</t>
         </is>
       </c>
       <c r="L41" s="7" t="inlineStr">
         <is>
-          <t>عدم حضور در کارتابل ۹ دارنده</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M41" s="12" t="n">
-        <v>0</v>
+        <v>56196200000</v>
       </c>
       <c r="N41" s="12" t="n">
-        <v>0</v>
+        <v>20803880000</v>
       </c>
       <c r="O41" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="P41" s="6" t="inlineStr"/>
+      <c r="P41" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-06 19:14:03</t>
+        </is>
+      </c>
       <c r="Q41" s="7" t="inlineStr">
         <is>
-          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 19:14:03 (کد پیگیری: 49686363364447)</t>
         </is>
       </c>
     </row>
@@ -6343,27 +6347,31 @@
       </c>
       <c r="K69" s="7" t="inlineStr">
         <is>
-          <t>علی رمضانزاده</t>
+          <t>مهدی زمانزاده</t>
         </is>
       </c>
       <c r="L69" s="7" t="inlineStr">
         <is>
-          <t>عدم حضور در کارتابل ۹ دارنده</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M69" s="12" t="n">
-        <v>0</v>
+        <v>28000000000</v>
       </c>
       <c r="N69" s="12" t="n">
-        <v>0</v>
+        <v>240000000</v>
       </c>
       <c r="O69" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="P69" s="6" t="inlineStr"/>
+      <c r="P69" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-06 19:14:03</t>
+        </is>
+      </c>
       <c r="Q69" s="7" t="inlineStr">
         <is>
-          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 19:14:03 (کد پیگیری: 49686363374741)</t>
         </is>
       </c>
     </row>
@@ -6416,27 +6424,31 @@
       </c>
       <c r="K70" s="11" t="inlineStr">
         <is>
-          <t>علی رمضانزاده</t>
+          <t>مهدی زمانزاده</t>
         </is>
       </c>
       <c r="L70" s="11" t="inlineStr">
         <is>
-          <t>عدم حضور در کارتابل ۹ دارنده</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M70" s="13" t="n">
-        <v>0</v>
+        <v>28000000000</v>
       </c>
       <c r="N70" s="13" t="n">
-        <v>0</v>
+        <v>240000000</v>
       </c>
       <c r="O70" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="P70" s="10" t="inlineStr"/>
+      <c r="P70" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-06 19:14:03</t>
+        </is>
+      </c>
       <c r="Q70" s="11" t="inlineStr">
         <is>
-          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 19:14:03 (کد پیگیری: 49686363377638)</t>
         </is>
       </c>
     </row>
@@ -8897,27 +8909,31 @@
       </c>
       <c r="K103" s="7" t="inlineStr">
         <is>
-          <t>علی رمضانزاده</t>
+          <t>مهدی زمانزاده</t>
         </is>
       </c>
       <c r="L103" s="7" t="inlineStr">
         <is>
-          <t>عدم حضور در کارتابل ۹ دارنده</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M103" s="12" t="n">
-        <v>0</v>
+        <v>48136400000</v>
       </c>
       <c r="N103" s="12" t="n">
-        <v>0</v>
+        <v>35000000</v>
       </c>
       <c r="O103" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="P103" s="6" t="inlineStr"/>
+      <c r="P103" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-06 19:14:03</t>
+        </is>
+      </c>
       <c r="Q103" s="7" t="inlineStr">
         <is>
-          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 19:14:03 (کد پیگیری: 49686363379579)</t>
         </is>
       </c>
     </row>
@@ -11641,27 +11657,31 @@
       </c>
       <c r="K139" s="7" t="inlineStr">
         <is>
-          <t>علی رمضانزاده</t>
+          <t>علیرضا ضیافتی</t>
         </is>
       </c>
       <c r="L139" s="7" t="inlineStr">
         <is>
-          <t>عدم حضور در کارتابل ۹ دارنده</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M139" s="12" t="n">
-        <v>0</v>
+        <v>93388000000</v>
       </c>
       <c r="N139" s="12" t="n">
-        <v>0</v>
+        <v>9840000000</v>
       </c>
       <c r="O139" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="P139" s="6" t="inlineStr"/>
+        <v>1326000000</v>
+      </c>
+      <c r="P139" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-06 19:14:03</t>
+        </is>
+      </c>
       <c r="Q139" s="7" t="inlineStr">
         <is>
-          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 19:14:03 (کد پیگیری: 49686363364456)</t>
         </is>
       </c>
     </row>
@@ -11714,27 +11734,31 @@
       </c>
       <c r="K140" s="11" t="inlineStr">
         <is>
-          <t>علی رمضانزاده</t>
+          <t>علیرضا ضیافتی</t>
         </is>
       </c>
       <c r="L140" s="11" t="inlineStr">
         <is>
-          <t>عدم حضور در کارتابل ۹ دارنده</t>
+          <t>استعلام زنده امروز (بروز)</t>
         </is>
       </c>
       <c r="M140" s="13" t="n">
-        <v>0</v>
+        <v>93388000000</v>
       </c>
       <c r="N140" s="13" t="n">
-        <v>0</v>
+        <v>9840000000</v>
       </c>
       <c r="O140" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P140" s="10" t="inlineStr"/>
+        <v>1326000000</v>
+      </c>
+      <c r="P140" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-06 19:14:03</t>
+        </is>
+      </c>
       <c r="Q140" s="11" t="inlineStr">
         <is>
-          <t>در استعلام گروهی امروز بررسی شد ولی در کارتابل هیچ‌یک از ۹ دارنده یافت نشد</t>
+          <t>استعلام زنده امروز درگاه پاسارگاد در ساعت 19:14:03 (کد پیگیری: 49686363379050)</t>
         </is>
       </c>
     </row>
@@ -13449,7 +13473,7 @@
         <v>3520000000</v>
       </c>
       <c r="J21" s="12" t="n">
-        <v>56196200000</v>
+        <v>112392400000</v>
       </c>
       <c r="K21" s="12" t="n">
         <v>0</v>
@@ -13730,7 +13754,7 @@
         </is>
       </c>
       <c r="E27" s="6" t="n">
-        <v>91.90000000000001</v>
+        <v>96</v>
       </c>
       <c r="F27" s="24" t="inlineStr">
         <is>
@@ -13749,7 +13773,7 @@
         <v>24000000000</v>
       </c>
       <c r="J27" s="12" t="n">
-        <v>252000000000</v>
+        <v>308000000000</v>
       </c>
       <c r="K27" s="12" t="n">
         <v>0</v>
@@ -14314,7 +14338,7 @@
         </is>
       </c>
       <c r="E39" s="6" t="n">
-        <v>25</v>
+        <v>29.2</v>
       </c>
       <c r="F39" s="23" t="inlineStr">
         <is>
@@ -14333,7 +14357,7 @@
         <v>16450000000</v>
       </c>
       <c r="J39" s="12" t="n">
-        <v>285933600000</v>
+        <v>334070000000</v>
       </c>
       <c r="K39" s="12" t="n">
         <v>1326000000</v>
@@ -14814,7 +14838,7 @@
         </is>
       </c>
       <c r="E49" s="6" t="n">
-        <v>20.7</v>
+        <v>0.6</v>
       </c>
       <c r="F49" s="23" t="inlineStr">
         <is>
@@ -14833,10 +14857,10 @@
         <v>22000000000</v>
       </c>
       <c r="J49" s="12" t="n">
-        <v>186776000000</v>
+        <v>373552000000</v>
       </c>
       <c r="K49" s="12" t="n">
-        <v>2652000000</v>
+        <v>5304000000</v>
       </c>
       <c r="L49" s="7" t="inlineStr">
         <is>

</xml_diff>